<commit_message>
feat: 新增 5 条 UI 测试覆盖（90% → 94%）— IPC mock 增强
增强 conftest mock：
- 新增 IPC 调用日志（window.__E2E_IPC_LOG__）供测试断言
- 新增动态覆盖机制（window.__E2E_IPC_OVERRIDES__）
- 补充 restore_ai_response、create_clipboard_workspace 等 mock 返回值

新增 Pytest 测试：
- test_restore_advanced.py: R02 AI回复还原（3 tests）、R04 历史还原（2 tests）
- test_workspace_advanced.py: W04 工作区配置隔离（3 tests）、W05 剪贴板工作区（2 tests）
- test_type_persistence.py: T13 enabled_types 持久化（3 tests）

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/testcases.xlsx
+++ b/e2e/testcases.xlsx
@@ -2597,21 +2597,21 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>未覆盖</t>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 17:48</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2711,21 +2711,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>未覆盖</t>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>部分覆盖</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 17:48</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3163,21 +3163,21 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>未覆盖</t>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="n"/>
-      <c r="N44" s="2" t="n"/>
-      <c r="O44" s="2" t="n"/>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 17:48</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3216,21 +3216,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>未覆盖</t>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="n"/>
-      <c r="N45" s="2" t="n"/>
-      <c r="O45" s="2" t="n"/>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 17:48</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7091,9 +7091,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="I104" s="2" t="inlineStr">
-        <is>
-          <t>未覆盖</t>
+      <c r="I104" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr"/>
@@ -7102,14 +7102,14 @@
           <t>持久化: enabled_types 保存和恢复</t>
         </is>
       </c>
-      <c r="L104" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M104" s="2" t="n"/>
-      <c r="N104" s="2" t="n"/>
-      <c r="O104" s="2" t="n"/>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 17:48</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: baseline 断言收紧为 hard+soft 全必中，新增 check_baseline 辅助
- assert_baseline: soft_missing 也计入失败
- format_baseline_report: 区分正则类 / NER 类未命中
- check_baseline: 一步完成断言 + 报告输出
- 新增真端到端测试计划文档

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/testcases.xlsx
+++ b/e2e/testcases.xlsx
@@ -660,7 +660,7 @@
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O2" s="2" t="n"/>
@@ -729,7 +729,7 @@
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O3" s="2" t="n"/>
@@ -800,7 +800,7 @@
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O4" s="2" t="n"/>
@@ -872,7 +872,7 @@
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O5" s="2" t="n"/>
@@ -940,12 +940,12 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>PDFium 动态库未部署(环境问题)</t>
+          <t>ENV-001: PDFium 动态库未部署</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
@@ -1011,15 +1011,19 @@
           <t>需创建加密 fixture</t>
         </is>
       </c>
-      <c r="L7" s="8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>BUG-020: 错误密码解密返回格式检测错误而非密码错误</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
@@ -1088,12 +1092,12 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>test_encrypted_xlsx_wrong_password: 密码错误重试测试失败</t>
+          <t>BUG-020: 错误密码解密返回格式检测错误而非密码错误</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
@@ -1156,15 +1160,19 @@
           <t>需创建空 fixture</t>
         </is>
       </c>
-      <c r="L9" s="8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>BUG-020: 错误密码解密返回格式检测错误而非密码错误</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
@@ -1227,15 +1235,19 @@
           <t>需创建大文件 fixture</t>
         </is>
       </c>
-      <c r="L10" s="8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>BUG-020: 错误密码解密返回格式检测错误而非密码错误</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
@@ -1306,7 +1318,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
@@ -1373,7 +1385,7 @@
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
@@ -1440,7 +1452,7 @@
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
@@ -1508,7 +1520,7 @@
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
@@ -1575,7 +1587,7 @@
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
@@ -1640,7 +1652,7 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
@@ -1708,7 +1720,7 @@
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
@@ -1776,7 +1788,7 @@
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
@@ -1845,7 +1857,7 @@
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
@@ -1913,7 +1925,7 @@
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
@@ -1980,7 +1992,7 @@
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
@@ -2047,7 +2059,7 @@
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
@@ -2114,7 +2126,7 @@
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
@@ -2181,7 +2193,7 @@
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
@@ -2248,7 +2260,7 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
@@ -2315,7 +2327,7 @@
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
@@ -2380,7 +2392,7 @@
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
@@ -2445,7 +2457,7 @@
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
@@ -2510,7 +2522,7 @@
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
@@ -2699,7 +2711,7 @@
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr"/>
@@ -2772,7 +2784,7 @@
       <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr"/>
@@ -2840,7 +2852,7 @@
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr"/>
@@ -2905,7 +2917,7 @@
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr"/>
@@ -2970,7 +2982,7 @@
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr"/>
@@ -3035,7 +3047,7 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr"/>
@@ -3100,7 +3112,7 @@
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr"/>
@@ -3222,7 +3234,7 @@
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr"/>
@@ -3287,7 +3299,7 @@
       <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr"/>
@@ -3348,7 +3360,7 @@
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr"/>
@@ -3409,7 +3421,7 @@
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr"/>
@@ -3469,12 +3481,12 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>IPC mock 返回 2 个工作区但列表只显示 1 个</t>
+          <t>BUG-019: 工作区列表渲染竞态</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr"/>
@@ -3527,15 +3539,19 @@
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>BUG-019: 工作区列表渲染竞态</t>
+        </is>
+      </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr"/>
@@ -3596,7 +3612,7 @@
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr"/>
@@ -3661,7 +3677,7 @@
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr"/>
@@ -3722,7 +3738,7 @@
       <c r="M48" s="2" t="inlineStr"/>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr"/>
@@ -3783,7 +3799,7 @@
       <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr"/>
@@ -3854,7 +3870,7 @@
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr"/>
@@ -3925,7 +3941,7 @@
       <c r="M51" s="2" t="inlineStr"/>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr"/>
@@ -3996,7 +4012,7 @@
       <c r="M52" s="2" t="inlineStr"/>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:48</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr"/>
@@ -4067,7 +4083,7 @@
       <c r="M53" s="2" t="inlineStr"/>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr"/>
@@ -4138,7 +4154,7 @@
       <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr"/>
@@ -4209,7 +4225,7 @@
       <c r="M55" s="2" t="inlineStr"/>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr"/>
@@ -4280,7 +4296,7 @@
       <c r="M56" s="2" t="inlineStr"/>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O56" s="2" t="inlineStr"/>
@@ -4351,7 +4367,7 @@
       <c r="M57" s="2" t="inlineStr"/>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O57" s="2" t="inlineStr"/>
@@ -4422,7 +4438,7 @@
       <c r="M58" s="2" t="inlineStr"/>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O58" s="2" t="inlineStr"/>
@@ -4493,7 +4509,7 @@
       <c r="M59" s="2" t="inlineStr"/>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O59" s="2" t="inlineStr"/>
@@ -4564,7 +4580,7 @@
       <c r="M60" s="2" t="inlineStr"/>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O60" s="2" t="inlineStr"/>
@@ -4635,7 +4651,7 @@
       <c r="M61" s="2" t="inlineStr"/>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O61" s="2" t="inlineStr"/>
@@ -4706,7 +4722,7 @@
       <c r="M62" s="2" t="inlineStr"/>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr"/>
@@ -4777,7 +4793,7 @@
       <c r="M63" s="2" t="inlineStr"/>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O63" s="2" t="inlineStr"/>
@@ -4848,7 +4864,7 @@
       <c r="M64" s="2" t="inlineStr"/>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr"/>
@@ -4919,7 +4935,7 @@
       <c r="M65" s="2" t="inlineStr"/>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr"/>
@@ -4990,7 +5006,7 @@
       <c r="M66" s="2" t="inlineStr"/>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr"/>
@@ -5061,7 +5077,7 @@
       <c r="M67" s="2" t="inlineStr"/>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O67" s="2" t="inlineStr"/>
@@ -5132,7 +5148,7 @@
       <c r="M68" s="2" t="inlineStr"/>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O68" s="2" t="inlineStr"/>
@@ -5203,7 +5219,7 @@
       <c r="M69" s="2" t="inlineStr"/>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O69" s="2" t="inlineStr"/>
@@ -5274,7 +5290,7 @@
       <c r="M70" s="2" t="inlineStr"/>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr"/>
@@ -5344,7 +5360,7 @@
       <c r="M71" s="2" t="inlineStr"/>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O71" s="2" t="inlineStr"/>
@@ -5414,7 +5430,7 @@
       <c r="M72" s="2" t="inlineStr"/>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr"/>
@@ -5483,12 +5499,12 @@
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>GBK 编码 CSV 解析失败，csv crate 仅支持 UTF-8</t>
+          <t>BUG-014: GBK 编码 CSV 解析失败，csv crate 仅支持 UTF-8</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O73" s="2" t="inlineStr"/>
@@ -5550,15 +5566,19 @@
           <t>测试 BOM 头处理</t>
         </is>
       </c>
-      <c r="L74" s="8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="M74" s="2" t="inlineStr"/>
+      <c r="L74" s="6" t="inlineStr">
+        <is>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>BUG-014: GBK 编码 CSV 解析失败，csv crate 仅支持 UTF-8</t>
+        </is>
+      </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O74" s="2" t="inlineStr"/>
@@ -5620,15 +5640,19 @@
           <t>全角数字 edge case</t>
         </is>
       </c>
-      <c r="L75" s="8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="M75" s="2" t="inlineStr"/>
+      <c r="L75" s="6" t="inlineStr">
+        <is>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>BUG-014: GBK 编码 CSV 解析失败，csv crate 仅支持 UTF-8</t>
+        </is>
+      </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O75" s="2" t="inlineStr"/>
@@ -5698,7 +5722,7 @@
       <c r="M76" s="2" t="inlineStr"/>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O76" s="2" t="inlineStr"/>
@@ -5768,7 +5792,7 @@
       <c r="M77" s="2" t="inlineStr"/>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O77" s="2" t="inlineStr"/>
@@ -5830,15 +5854,19 @@
           <t>超大单元格性能和准确性</t>
         </is>
       </c>
-      <c r="L78" s="8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="M78" s="2" t="inlineStr"/>
+      <c r="L78" s="6" t="inlineStr">
+        <is>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>BUG-014: GBK 编码 CSV 解析失败，csv crate 仅支持 UTF-8</t>
+        </is>
+      </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O78" s="2" t="inlineStr"/>
@@ -5908,7 +5936,7 @@
       <c r="M79" s="2" t="inlineStr"/>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O79" s="2" t="inlineStr"/>
@@ -5974,7 +6002,7 @@
       <c r="M80" s="2" t="inlineStr"/>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O80" s="2" t="inlineStr"/>
@@ -6040,7 +6068,7 @@
       <c r="M81" s="2" t="inlineStr"/>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O81" s="2" t="inlineStr"/>
@@ -6110,7 +6138,7 @@
       <c r="M82" s="2" t="inlineStr"/>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O82" s="2" t="inlineStr"/>
@@ -6176,7 +6204,7 @@
       <c r="M83" s="2" t="inlineStr"/>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O83" s="2" t="inlineStr"/>
@@ -6246,7 +6274,7 @@
       <c r="M84" s="2" t="inlineStr"/>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O84" s="2" t="inlineStr"/>
@@ -6312,7 +6340,7 @@
       <c r="M85" s="2" t="inlineStr"/>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O85" s="2" t="inlineStr"/>
@@ -6382,7 +6410,7 @@
       <c r="M86" s="2" t="inlineStr"/>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O86" s="2" t="inlineStr"/>
@@ -6453,7 +6481,7 @@
       <c r="M87" s="2" t="inlineStr"/>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O87" s="2" t="inlineStr"/>
@@ -6524,7 +6552,7 @@
       <c r="M88" s="2" t="inlineStr"/>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O88" s="2" t="inlineStr"/>
@@ -6586,13 +6614,17 @@
           <t>错误隔离</t>
         </is>
       </c>
-      <c r="L89" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M89" s="2" t="n"/>
-      <c r="N89" s="2" t="n"/>
+      <c r="L89" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr"/>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 23:15</t>
+        </is>
+      </c>
       <c r="O89" s="2" t="n"/>
     </row>
     <row r="90">
@@ -6652,13 +6684,17 @@
           <t>中文列名匹配</t>
         </is>
       </c>
-      <c r="L90" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M90" s="2" t="n"/>
-      <c r="N90" s="2" t="n"/>
+      <c r="L90" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr"/>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 23:15</t>
+        </is>
+      </c>
       <c r="O90" s="2" t="n"/>
     </row>
     <row r="91">
@@ -6718,13 +6754,17 @@
           <t>英文列名匹配</t>
         </is>
       </c>
-      <c r="L91" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M91" s="2" t="n"/>
-      <c r="N91" s="2" t="n"/>
+      <c r="L91" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr"/>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 23:15</t>
+        </is>
+      </c>
       <c r="O91" s="2" t="n"/>
     </row>
     <row r="92">
@@ -6793,7 +6833,7 @@
       <c r="M92" s="2" t="inlineStr"/>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O92" s="2" t="inlineStr"/>
@@ -6860,7 +6900,7 @@
       <c r="M93" s="2" t="inlineStr"/>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O93" s="2" t="inlineStr"/>
@@ -6919,13 +6959,17 @@
           <t>主题切换</t>
         </is>
       </c>
-      <c r="L94" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M94" s="2" t="n"/>
-      <c r="N94" s="2" t="n"/>
+      <c r="L94" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr"/>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 23:15</t>
+        </is>
+      </c>
       <c r="O94" s="2" t="n"/>
     </row>
     <row r="95">
@@ -6983,13 +7027,17 @@
           <t>本地存储持久化</t>
         </is>
       </c>
-      <c r="L95" s="2" t="inlineStr">
-        <is>
-          <t>未执行</t>
-        </is>
-      </c>
-      <c r="M95" s="2" t="n"/>
-      <c r="N95" s="2" t="n"/>
+      <c r="L95" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04 23:15</t>
+        </is>
+      </c>
       <c r="O95" s="2" t="n"/>
     </row>
     <row r="96">
@@ -7058,12 +7106,12 @@
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>UkPhone +44 161 496 0000(含空格格式)未被正则识别</t>
+          <t>BUG-015: UkPhone 含空格格式未识别</t>
         </is>
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O96" s="2" t="inlineStr"/>
@@ -7134,12 +7182,12 @@
       </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>DriversLicense S012-3456-7890 未识别</t>
+          <t>BUG-016: DriversLicense S开头格式未识别</t>
         </is>
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O97" s="2" t="inlineStr"/>
@@ -7210,12 +7258,12 @@
       </c>
       <c r="M98" s="2" t="inlineStr">
         <is>
-          <t>Passport 号码完全未识别(0/3)，国际驾照格式缺失</t>
+          <t>BUG-017: Passport 和国际驾照格式正则缺失</t>
         </is>
       </c>
       <c r="N98" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O98" s="2" t="inlineStr"/>
@@ -7287,7 +7335,7 @@
       <c r="M99" s="2" t="inlineStr"/>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O99" s="2" t="inlineStr"/>
@@ -7359,7 +7407,7 @@
       <c r="M100" s="2" t="inlineStr"/>
       <c r="N100" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O100" s="2" t="inlineStr"/>
@@ -7431,7 +7479,7 @@
       <c r="M101" s="2" t="inlineStr"/>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O101" s="2" t="inlineStr"/>
@@ -7502,7 +7550,7 @@
       <c r="M102" s="2" t="inlineStr"/>
       <c r="N102" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O102" s="2" t="inlineStr"/>
@@ -7574,7 +7622,7 @@
       <c r="M103" s="2" t="inlineStr"/>
       <c r="N103" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O103" s="2" t="inlineStr"/>
@@ -7645,12 +7693,12 @@
       </c>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>IPC mock selectWorkspace 未正确触发 store 更新</t>
+          <t>BUG-018: IPC mock enabled_types 为 null</t>
         </is>
       </c>
       <c r="N104" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O104" s="2" t="inlineStr"/>
@@ -7721,7 +7769,7 @@
       <c r="M105" s="2" t="inlineStr"/>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O105" s="2" t="inlineStr"/>
@@ -7791,7 +7839,7 @@
       <c r="M106" s="2" t="inlineStr"/>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O106" s="2" t="inlineStr"/>
@@ -7862,7 +7910,7 @@
       <c r="M107" s="2" t="inlineStr"/>
       <c r="N107" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O107" s="2" t="inlineStr"/>
@@ -7933,7 +7981,7 @@
       <c r="M108" s="2" t="inlineStr"/>
       <c r="N108" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04 21:49</t>
+          <t>2026-04-04 23:15</t>
         </is>
       </c>
       <c r="O108" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
test(excel): 补回远程 13 个用例 — C80/C81/S23-S31/K09/B14
rebase 时为保留本地 B06-B13 批量场景而选用了本地 xlsx，丢失了远程在
312b0b9 / 3b47b56 中新增的 13 个用例（英文 Replace 策略 S23-S31、
英文管道 C80/C81、中英 counter 隔离 K09、英文批量 NER B14）。

本次手动比对三个版本（base b23f703、远程 312b0b9、本地 current）后
将远程独有用例追加到末尾，远程 B06 与本地 B06 语义不同，重命名为
B14 共存。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/testcases.xlsx
+++ b/e2e/testcases.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixture数据基线" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖率统计" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fixture数据基线" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="覆盖率统计" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$O$49</definedName>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O178"/>
+  <dimension ref="A1:O191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12851,6 +12851,892 @@
         </is>
       </c>
       <c r="O178" s="2" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>C80</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>核心管道</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>英文文档完整管道 — 三路识别 + Replace 替换全链路验证</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 模型已加载；fixture 含至少 4 个英文 PersonName/OrgName/Address/Title</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 调 detect_by_regex / detect_by_dict / detect_by_ner 三路识别
+3. 收集 NER items 中的 4 类 NER 实体（PersonName/OrgName/Address/Title）
+4. 配 Strategy::Replace { Fake } 调 apply_desensitize
+5. 检查 — 对 NER 识别到的每个实体，其原文在脱敏后文档中不再出现</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>ner_items.len() &gt; 0（NER 必须有产出，不能因加载失败被吞掉）；对 NER 识别到的每一个 PersonName/OrgName/Address/Title item，脱敏后文档中不再包含 item.text 原文（即真的发生了替换）；替换后输出全部不含汉字。注：本用例验证'真的发生了替换'这一功能 bug，不验证 NER 召回率（distilbert-ner 在法律文书上召回率约 60-80%，未识别的实体保持原文是模型限制非 bug）</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I179" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>full_pipeline_english.rs</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="n"/>
+      <c r="L179" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M179" s="2" t="n"/>
+      <c r="N179" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O179" s="2" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Fake — PersonName 输出含空格、纯 ASCII、不含汉字</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 已识别出 4 个英文 PersonName（James Anderson 等）</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 三路识别后筛 PersonName items
+3. 配 Strategy::Replace { style: Fake } 调 apply_desensitize
+4. 取每个 PersonName 替换后的输出</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>每个替换值满足：(a) 不含汉字 (b) 含空格分隔 First Last (c) 不等于原文 (d) 不是 'John Doe'/'Jane Doe'（那是 Mou 占位）</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I180" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="n"/>
+      <c r="L180" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M180" s="2" t="n"/>
+      <c r="N180" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O180" s="2" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Fake — OrgName 输出以 EN 字典 suffix 结尾</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 已识别出 4 个英文 OrgName</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 筛 OrgName items
+3. 配 Strategy::Replace { style: Fake }
+4. 校验每个替换值末尾的 suffix</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>每个替换值末尾 ∈ EN_ORG_SUFFIXES (Inc./Corp./LLC/LLP/Ltd./Group/Holdings/Partners/Associates/International/Co.)；不含汉字；不等于原文</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I181" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="n"/>
+      <c r="L181" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M181" s="2" t="n"/>
+      <c r="N181" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O181" s="2" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Fake — Address 输出含逗号、不含汉字</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 已识别出 3 个英文 Address</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 筛 Address items
+3. 配 Strategy::Replace { style: Fake }
+4. 校验每个替换值的形态</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>每个替换值满足：(a) 不含汉字 (b) 形如 '&lt;number&gt; &lt;street&gt;, &lt;city&gt;'（含至少一个逗号分隔街道与城市）(c) 不等于原文</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I182" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="n"/>
+      <c r="L182" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M182" s="2" t="n"/>
+      <c r="N182" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O182" s="2" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>S26</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Fake — Title 输出在英文 titles 池内</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 已识别出 3 种英文 Title (Senior Partner / Associate Attorney / Managing Partner)</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 筛 Title items
+3. 配 Strategy::Replace { style: Fake }
+4. 校验每个替换值</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>每个替换值满足：(a) 不含汉字 (b) 在 fake_data/en/titles.json 池内（或附 wrap 后缀）(c) 不等于原文</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I183" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K183" s="2" t="n"/>
+      <c r="L183" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M183" s="2" t="n"/>
+      <c r="N183" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O183" s="2" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Mou — PersonName 性别轮换 John Doe / Jane Doe / John Doe 2 / Jane Doe 2</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 已识别出 4 个英文 PersonName；Strategy::Replace 默认 consistent: true，即同一原文复用替换值，4 个 unique 原文消费 4 次 mou_name_en counter</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 三路识别 → 筛 PersonName items，按 unique 原文聚合
+3. 配 Strategy::Replace { style: Mou }
+4. 取每个 unique PersonName 的替换值，组成集合</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>4 个 unique PersonName 替换值集合 == {'John Doe', 'Jane Doe', 'John Doe 2', 'Jane Doe 2'}；用集合断言（不依赖 NER items 出现顺序），覆盖性别二选一轮换 + 第 N 对加序号的契约</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I184" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="n"/>
+      <c r="L184" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="n"/>
+      <c r="N184" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O184" s="2" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>S28</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Mou — OrgName 保留原文 suffix，无 suffix 兜底 Acme Co.</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；fixture 含 4 个 OrgName: Mitchell, Chen &amp; Park LLP / Pacific Coast Medical Center / Harrison &amp; Associates LLP / TechVenture Capital Partners；其中 LLP 命中表（第 1+2 次）、Partners 命中表（第 1 次）、Center 不在表（走兜底）</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 三路识别 → 筛 OrgName items，按 unique 原文聚合
+3. 配 Strategy::Replace { style: Mou }
+4. 取每个 unique OrgName 的替换值，组成集合</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>4 个 unique OrgName 替换值集合 == {'Acme Partners', 'Acme LLP', 'Acme LLP 2', 'Acme Co.'}；TechVenture Capital Partners → 'Acme Partners'（命中 Partners suffix，counter mou_org_en_Partners=1）；Mitchell, Chen &amp; Park LLP → 'Acme LLP'（counter mou_org_en_LLP=1）；Harrison &amp; Associates LLP → 'Acme LLP 2'（counter mou_org_en_LLP=2）；Pacific Coast Medical Center → 'Acme Co.'（末尾 Center 不在 EN_ORG_SUFFIXES，走兜底，counter mou_org_en_Co.=1）</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I185" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="n"/>
+      <c r="L185" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M185" s="2" t="n"/>
+      <c r="N185" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Mou — Address 输出 [REDACTED CITY] 序号化</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 已识别出 3 个英文 Address</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 筛 Address items（按出现顺序）
+3. 配 Strategy::Replace { style: Mou }
+4. 校验替换值序列</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>前 3 个 unique Address 替换值依次为：'[REDACTED CITY]', '[REDACTED CITY] 2', '[REDACTED CITY] 3'</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I186" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="n"/>
+      <c r="L186" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="n"/>
+      <c r="N186" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O186" s="2" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>S30</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Mou — Title 输出 [REDACTED TITLE] 序号化</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；NER 已识别出 3 种英文 Title</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 筛 Title items（按 unique 原文）
+3. 配 Strategy::Replace { style: Mou }
+4. 校验替换值序列</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>前 3 个 unique Title 替换值依次为：'[REDACTED TITLE]', '[REDACTED TITLE] 2', '[REDACTED TITLE] 3'</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I187" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="n"/>
+      <c r="L187" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M187" s="2" t="n"/>
+      <c r="N187" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O187" s="2" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>S31</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>策略切换</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>EN Replace Ordinal — 静默降级为 Fake，不输出 'Person A' / 'Company A' / 'Address 1' / 'Title 1'</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage=En；同 fixture 4 类 NER 实体齐全</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 attorney_engagement_letter.docx
+2. 三路识别
+3. 4 类 NER 实体配 Strategy::Replace { style: Ordinal }
+4. 取每个 NER 实体的 Ordinal 输出，断言形态等同 Fake（即降级生效，未输出 'Person A' 这类原始 ordinal 形态）</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>PersonName 输出含空格、不以 'Person ' 开头；OrgName 输出末尾在 EN_ORG_SUFFIXES、不以 'Company ' 开头；Address 输出含逗号、不以 'Address ' 开头；Title 输出不以 'Title ' 开头；所有输出不含汉字（即降级为 Fake 等效行为）</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I188" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>strategy_switching_en_replace.rs</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="n"/>
+      <c r="L188" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M188" s="2" t="n"/>
+      <c r="N188" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>K09</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>一致性替换</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>中英 counter 隔离 — 文档含中英混合 PersonName，counter 中独立计数 PersonName_zh + PersonName_en</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>AppLanguage 任意（替换走 apply_replace 内部 detect_language(text) 自动判断，不依赖 AppLanguage）；fixture mixed_bilingual.xlsx baseline 标注 4 个中文 PersonName + 4 个英文 PersonName；实际 NER 识别数依赖模型（当前 distilbert-ner 对中文识别可能为零，因此本用例的语义聚焦于'识别到的部分如何分桶'，不强求识别完整性</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>1. 导入 mixed_bilingual.xlsx
+2. 三路识别 → 8 个 PersonName items（4 中 4 英）
+3. 配 Strategy::Replace { style: Fake } 调 apply_desensitize（开启 consistent，绑定工作区以触发 counter 持久化）
+4. 读 workspace.replace_counters，检查 PersonName_zh 与 PersonName_en 分别计数</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>对 NER 识别到的每个 PersonName item：含汉字 → 进 PersonName_zh counter；纯 ASCII → 进 PersonName_en counter；两个 counter 互不串扰；PersonName_zh + PersonName_en 之和 == apply_replace 实际消费次数（即所有识别出的 unique PersonName 数）；中文 item 替换值含汉字（来自中文 fake 池）；英文 item 替换值含空格、纯 ASCII（来自英文 fake 池）；若 NER 完全识别不出某语言（如英文模型识别不到中文），对应 counter 缺失或为 0 是模型问题非 bug</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/xlsx/mixed_bilingual.xlsx</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I189" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>consistency_bilingual.rs</t>
+        </is>
+      </c>
+      <c r="K189" s="2" t="n"/>
+      <c r="L189" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M189" s="2" t="n"/>
+      <c r="N189" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>C81</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>核心管道</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>英文文档在 NER degraded 模式下 — regex/dict 仍能识别替换 SSN/UsPhone/Email 等正则类型</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>测试路径：Rust 集成测试（tests/*.rs），通过构造 NerEngineState(Arc::new(Mutex::new(NerEngine::degraded()))) 注入降级引擎；AppLanguage=En；fixture 含 SSN/UsPhone/Email/CreditCard/Iban；前端 Tauri command 路径无法替换 NER 引擎，本用例不能走 Playwright e2e</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>1. 用 NerEngine::degraded() 替换 NER 引擎
+2. 导入 attorney_engagement_letter.docx
+3. 三路识别 — NER 应返回空，regex/dict 应正常
+4. SSN/UsPhone/Email/CreditCard/Iban 配 Strategy::Mask 调 apply_desensitize
+5. 检查脱敏后这些类型已被 Mask（带 *）</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>ner_items.len() == 0；regex_items.len() &gt; 0（识别到至少 SSN + UsPhone + Email）；脱敏后 SSN/UsPhone/Email 等正则类型在文档中已被 Mask 替换；PersonName/OrgName 等 NER 类型因未识别故保持原文（可接受降级行为，不是 bug）</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I190" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>full_pipeline_english.rs</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="n"/>
+      <c r="L190" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M190" s="2" t="n"/>
+      <c r="N190" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>B14</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>批量处理</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>批量脱敏 — 多个英文文档批处理后 NER 实体应被替换（覆盖用户报告的批量没替换 bug）</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>测试路径：Playwright e2e（e2e/tests/）— 走前端 useBatchAutoProcess Hook，更接近真实用户场景；或后端 Rust 集成测试 — 模拟批量调用 detect_by_* + apply_desensitize 串联；AppLanguage=En；NER 已加载；batch session 含 2 个英文 fixture (docx + xlsx)</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>1. 批量导入 attorney_engagement_letter.docx + law_firm_client_intake.xlsx
+2. 走 useBatchAutoProcess pipeline（regex + dict + NER 三路 + apply_desensitize）
+3. 检查每个文件的 desensitizeResult.summary.by_type
+4. 检查每个文件的 mappings 中包含 PersonName/OrgName 类型条目</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>批量结果中每个文件的 mappings 至少包含一条 PersonName 类型映射（即真的发生了 NER 替换）；脱敏后文档中所有 baseline PersonName 原文不存在；替换值符合英文 Fake 形态（含空格、纯 ASCII）；覆盖批量调用链路与单文件等价</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>scenarios/docx/attorney_engagement_letter.docx</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I191" s="8" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>batch_processing.rs</t>
+        </is>
+      </c>
+      <c r="K191" s="2" t="n"/>
+      <c r="L191" s="8" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M191" s="2" t="n"/>
+      <c r="N191" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:36</t>
+        </is>
+      </c>
+      <c r="O191" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O49"/>

</xml_diff>

<commit_message>
test(regression): 引入静默 passthrough 拦截网 + bundle 资源二次校验
- 新增 Rust/Python 双侧 regression helper，断言脱敏 content 真改、summary 不虚报
- scripts/verify-bundle.sh 校验 ONNX 模型 / pdfium 齐全，release 脚本前后两次拦截
- 新增 e2e/fixtures/regression/ 用户痛点 fixture 目录与示例 fixture
</commit_message>
<xml_diff>
--- a/e2e/testcases.xlsx
+++ b/e2e/testcases.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fixture数据基线" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="覆盖率统计" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixture数据基线" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖率统计" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$O$195</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fixture数据基线'!$A$1:$F$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +36,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -85,6 +85,12 @@
         <bgColor rgb="00D3F9D8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -133,6 +139,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O191"/>
+  <dimension ref="A1:O195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13738,8 +13748,296 @@
       </c>
       <c r="O191" s="2" t="n"/>
     </row>
+    <row r="192">
+      <c r="A192" s="10" t="inlineStr">
+        <is>
+          <t>C82</t>
+        </is>
+      </c>
+      <c r="B192" s="10" t="inlineStr">
+        <is>
+          <t>核心管道</t>
+        </is>
+      </c>
+      <c r="C192" s="10" t="inlineStr">
+        <is>
+          <t>防 silent passthrough — 单文件场景跨格式回归（用户痛点 #1）</t>
+        </is>
+      </c>
+      <c r="D192" s="10" t="inlineStr">
+        <is>
+          <t>NER 模型已加载；fixture sample.* 已存在；测试路径双侧覆盖：Rust 全管线集成测 + Playwright 前端管线 mock 测</t>
+        </is>
+      </c>
+      <c r="E192" s="10" t="inlineStr">
+        <is>
+          <t>1. 解析 fixture（xlsx/csv/docx/txt）
+2. 三路识别（regex + dict + NER）
+3. apply_desensitize 走 Replace+Fake
+4. 断言: result.content 与原文不同 + summary.total &gt; 0 + mappings 非空</t>
+        </is>
+      </c>
+      <c r="F192" s="10" t="inlineStr">
+        <is>
+          <t>脱敏后 content 与原文 flatten 文本严格不等（assert_ne!）；summary.total &gt; 0 且 mappings 数 ≥ summary.total/2；识别项数达到基线（xlsx/csv ≥ 20，docx/txt ≥ 8）；任一断言失败精确报告对应原因（漏识别 / 策略 noop / 静默 passthrough）</t>
+        </is>
+      </c>
+      <c r="G192" s="10" t="inlineStr">
+        <is>
+          <t>sample.xlsx, sample.csv, sample.docx, sample.txt</t>
+        </is>
+      </c>
+      <c r="H192" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I192" s="10" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J192" s="10" t="inlineStr">
+        <is>
+          <t>regression_no_passthrough.rs + e2e/tests/test_no_silent_passthrough.py</t>
+        </is>
+      </c>
+      <c r="K192" s="10" t="inlineStr">
+        <is>
+          <t>防止「测试都过但 UI 全部都没有替换」复发；新加 fixture 时复用 assert_no_silent_passthrough helper</t>
+        </is>
+      </c>
+      <c r="L192" s="10" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M192" s="11" t="n"/>
+      <c r="N192" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:56</t>
+        </is>
+      </c>
+      <c r="O192" s="11" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="10" t="inlineStr">
+        <is>
+          <t>C83</t>
+        </is>
+      </c>
+      <c r="B193" s="10" t="inlineStr">
+        <is>
+          <t>核心管道</t>
+        </is>
+      </c>
+      <c r="C193" s="10" t="inlineStr">
+        <is>
+          <t>前端脱敏管线 IPC 调用顺序与状态机完整性</t>
+        </is>
+      </c>
+      <c r="D193" s="10" t="inlineStr">
+        <is>
+          <t>Vite dev server 已起；__E2E_IPC_OVERRIDES__ 注入完整管线 mock；__DIMKEY_STORE__ 已暴露</t>
+        </is>
+      </c>
+      <c r="E193" s="10" t="inlineStr">
+        <is>
+          <t>1. 注入完整 mock（import_file + detect_by_* + apply_desensitize + add_processing_record）
+2. reset_ipc_log
+3. 调 window.__DIMKEY_PROCESS_FILE__
+4. 等待 view 切到 comparison
+5. 读 __E2E_IPC_LOG__ 与 store state</t>
+        </is>
+      </c>
+      <c r="F193" s="10" t="inlineStr">
+        <is>
+          <t>IPC 顺序: import_file &lt; detect_by_regex &lt; apply_desensitize &lt; add_processing_record；processingStep 终态为 'done'；centerView 终态为 'comparison'；store.currentResult 不为 null；summary.total 与 mappings.length 一致</t>
+        </is>
+      </c>
+      <c r="G193" s="10" t="inlineStr">
+        <is>
+          <t>sample.txt（mock 注入内容）</t>
+        </is>
+      </c>
+      <c r="H193" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I193" s="10" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J193" s="10" t="inlineStr">
+        <is>
+          <t>e2e/tests/test_no_silent_passthrough.py</t>
+        </is>
+      </c>
+      <c r="K193" s="10" t="inlineStr">
+        <is>
+          <t>覆盖前端 hook useAutoDesensitize 的状态机正确性；与 batch_auto 形成互补（B14 走批量路径）</t>
+        </is>
+      </c>
+      <c r="L193" s="10" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M193" s="11" t="n"/>
+      <c r="N193" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:56</t>
+        </is>
+      </c>
+      <c r="O193" s="11" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="10" t="inlineStr">
+        <is>
+          <t>C84</t>
+        </is>
+      </c>
+      <c r="B194" s="10" t="inlineStr">
+        <is>
+          <t>核心管道</t>
+        </is>
+      </c>
+      <c r="C194" s="10" t="inlineStr">
+        <is>
+          <t>Meta — 反向验证 silent passthrough 能被测试体系抓到</t>
+        </is>
+      </c>
+      <c r="D194" s="10" t="inlineStr">
+        <is>
+          <t>完整管线 mock 注入；apply_desensitize 故意返回 content === 原文（「假装替换了」）</t>
+        </is>
+      </c>
+      <c r="E194" s="10" t="inlineStr">
+        <is>
+          <t>1. 注入 silent_passthrough mock（apply_desensitize 返回 content 等于原文，但 summary.total = 1）
+2. 触发 processFile
+3. 等 view 切到 comparison
+4. 调 assert_desensitization_applied(min_replacements=1)</t>
+        </is>
+      </c>
+      <c r="F194" s="10" t="inlineStr">
+        <is>
+          <t>assert_desensitization_applied 必须 raise AssertionError，错误消息包含「脱敏后内容与原文完全相同」；这是断言体系的元测试 — 防止 helper 被误改后失去抓 bug 能力</t>
+        </is>
+      </c>
+      <c r="G194" s="10" t="inlineStr">
+        <is>
+          <t>sample.txt（mock 注入伪造结果）</t>
+        </is>
+      </c>
+      <c r="H194" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I194" s="10" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J194" s="10" t="inlineStr">
+        <is>
+          <t>e2e/tests/test_no_silent_passthrough.py::test_silent_passthrough_is_caught</t>
+        </is>
+      </c>
+      <c r="K194" s="10" t="inlineStr">
+        <is>
+          <t>Meta-test：测试用来验证测试本身。一旦某次 PR 改坏了 assert_desensitization_applied，本用例会立刻失败</t>
+        </is>
+      </c>
+      <c r="L194" s="10" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M194" s="11" t="n"/>
+      <c r="N194" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:56</t>
+        </is>
+      </c>
+      <c r="O194" s="11" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="10" t="inlineStr">
+        <is>
+          <t>PK01</t>
+        </is>
+      </c>
+      <c r="B195" s="10" t="inlineStr">
+        <is>
+          <t>发版打包</t>
+        </is>
+      </c>
+      <c r="C195" s="10" t="inlineStr">
+        <is>
+          <t>macOS Bundle 资源完整性 smoke check（用户痛点 #2）</t>
+        </is>
+      </c>
+      <c r="D195" s="10" t="inlineStr">
+        <is>
+          <t>已执行 cargo tauri build；产物在 src-tauri/target/release/bundle/macos/Dimkey.app；脚本依赖 stat / hdiutil（macOS 自带）</t>
+        </is>
+      </c>
+      <c r="E195" s="10" t="inlineStr">
+        <is>
+          <t>1. 跑 ./scripts/verify-bundle.sh &lt;Dimkey.app&gt; macos
+2. 检查 4 项: ner/model.onnx ≥ 30MB; ner/tokenizer.json + id2label.json + model_config.json 全在; pdfium/libpdfium.dylib ≥ 1MB; Contents/MacOS/Dimkey 可执行
+3. release-macos.sh 自动调用 build 后 + tar.gz 解压后 + DMG 挂载后三处校验</t>
+        </is>
+      </c>
+      <c r="F195" s="10" t="inlineStr">
+        <is>
+          <t>任一资源缺失或体积异常 → exit 1 拒绝发布；脚本在 release-macos.sh 三个挂钩点都跑（避免打包过程丢失）；DMG 校验通过 hdiutil attach 临时挂载实现</t>
+        </is>
+      </c>
+      <c r="G195" s="10" t="inlineStr">
+        <is>
+          <t>n/a（校验对象为构建产物本身）</t>
+        </is>
+      </c>
+      <c r="H195" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I195" s="10" t="inlineStr">
+        <is>
+          <t>已覆盖</t>
+        </is>
+      </c>
+      <c r="J195" s="10" t="inlineStr">
+        <is>
+          <t>scripts/verify-bundle.sh + scripts/release-macos.sh</t>
+        </is>
+      </c>
+      <c r="K195" s="10" t="inlineStr">
+        <is>
+          <t>首次跑就抓到当前 src-tauri/resources/pdfium/ 只有 .gitkeep 的真实 bug；防止「打包后模型文件都没带」复发</t>
+        </is>
+      </c>
+      <c r="L195" s="10" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="M195" s="11" t="n"/>
+      <c r="N195" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:56</t>
+        </is>
+      </c>
+      <c r="O195" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O49"/>
+  <autoFilter ref="A1:O195"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -54200,7 +54498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -54246,272 +54544,296 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>核心管道</t>
+          <t>UI交互</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="E2" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>4/9 (部分)</t>
+          <t>5/6</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>策略切换</t>
+          <t>一致性替换</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>7/9</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>类型过滤</t>
+          <t>列级规则</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="n">
         <v>4</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>4/6</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>字典/白名单</t>
+          <t>发版打包</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>1/1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>列级规则</t>
+          <t>字典/白名单</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>10/10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>一致性替换</t>
+          <t>工作区管理</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>5/6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>还原</t>
+          <t>批量处理</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="E8" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1/4 (部分)</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>批量处理</t>
+          <t>核心管道</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>84/84</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>工作区管理</t>
+          <t>策略切换</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C10" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="E10" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1/5 (部分)</t>
+          <t>31/31</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UI交互</t>
+          <t>类型过滤</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>21/21</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>还原</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>7/48 (14.6%)</t>
+      <c r="B14" t="n">
+        <v>194</v>
+      </c>
+      <c r="C14" t="n">
+        <v>186</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>186/194 (95.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>